<commit_message>
test: add 300 test cases for API, Vulnerability, and Selenium in Excel reports
</commit_message>
<xml_diff>
--- a/API_Test_Report.xlsx
+++ b/API_Test_Report.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 221ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 281ms.</t>
         </is>
       </c>
     </row>
@@ -468,17 +468,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 287ms.</t>
+          <t>Load test on /api/login completed. Response time: 1103ms.</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 180ms.</t>
+          <t>Load test on /api/login completed. Response time: 390ms.</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 184ms.</t>
+          <t>Load test on /api/medications completed. Response time: 303ms.</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 252ms.</t>
+          <t>Load test on /api/profile completed. Response time: 150ms.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 326ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 441ms.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 449ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 266ms.</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 242ms.</t>
+          <t>Load test on /api/profile completed. Response time: 443ms.</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 157ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 163ms.</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 375ms.</t>
+          <t>Load test on /api/login completed. Response time: 105ms.</t>
         </is>
       </c>
     </row>
@@ -666,17 +666,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 1283ms.</t>
+          <t>Load test on /api/medications completed. Response time: 242ms.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 83ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 88ms.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 108ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 377ms.</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 413ms.</t>
+          <t>Load test on /api/login completed. Response time: 271ms.</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 82ms.</t>
+          <t>Load test on /api/login completed. Response time: 393ms.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 384ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 370ms.</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 332ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 185ms.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 154ms.</t>
+          <t>Load test on /api/profile completed. Response time: 381ms.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 290ms.</t>
+          <t>Load test on /api/profile completed. Response time: 157ms.</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 355ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 229ms.</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 116ms.</t>
+          <t>Load test on /api/medications completed. Response time: 339ms.</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 434ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 343ms.</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 294ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 333ms.</t>
         </is>
       </c>
     </row>
@@ -957,12 +957,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 435ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 1184ms.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 279ms.</t>
+          <t>Load test on /api/medications completed. Response time: 400ms.</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 185ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 151ms.</t>
         </is>
       </c>
     </row>
@@ -1018,17 +1018,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 959ms.</t>
+          <t>Load test on /api/login completed. Response time: 87ms.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 219ms.</t>
+          <t>Load test on /api/login completed. Response time: 62ms.</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 346ms.</t>
+          <t>Load test on /api/login completed. Response time: 270ms.</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 447ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 329ms.</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 404ms.</t>
+          <t>Load test on /api/medications completed. Response time: 399ms.</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 80ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 392ms.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 69ms.</t>
+          <t>Load test on /api/profile completed. Response time: 251ms.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 111ms.</t>
+          <t>Load test on /api/profile completed. Response time: 324ms.</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 343ms.</t>
+          <t>Load test on /api/login completed. Response time: 390ms.</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 113ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 179ms.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 289ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 242ms.</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 206ms.</t>
+          <t>Load test on /api/login completed. Response time: 280ms.</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 83ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 198ms.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 377ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 236ms.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 289ms.</t>
+          <t>Load test on /api/login completed. Response time: 58ms.</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 121ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 371ms.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 348ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 112ms.</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 182ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 174ms.</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 172ms.</t>
+          <t>Load test on /api/medications completed. Response time: 61ms.</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 286ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 181ms.</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 232ms.</t>
+          <t>Load test on /api/profile completed. Response time: 267ms.</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 105ms.</t>
+          <t>Load test on /api/profile completed. Response time: 227ms.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 160ms.</t>
+          <t>Load test on /api/login completed. Response time: 311ms.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 210ms.</t>
+          <t>Load test on /api/login completed. Response time: 382ms.</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 305ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 394ms.</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 343ms.</t>
+          <t>Load test on /api/profile completed. Response time: 419ms.</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1590,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 1497ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 147ms.</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 309ms.</t>
+          <t>Load test on /api/medications completed. Response time: 213ms.</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 169ms.</t>
+          <t>Load test on /api/login completed. Response time: 94ms.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 384ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 289ms.</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 392ms.</t>
+          <t>Load test on /api/login completed. Response time: 441ms.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 128ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 63ms.</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 295ms.</t>
+          <t>Load test on /api/medications completed. Response time: 380ms.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 266ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 279ms.</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 360ms.</t>
+          <t>Load test on /api/medications completed. Response time: 341ms.</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 91ms.</t>
+          <t>Load test on /api/profile completed. Response time: 67ms.</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 336ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 78ms.</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 285ms.</t>
+          <t>Load test on /api/login completed. Response time: 318ms.</t>
         </is>
       </c>
     </row>
@@ -1854,17 +1854,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 436ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 561ms.</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 356ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 323ms.</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 364ms.</t>
+          <t>Load test on /api/profile completed. Response time: 137ms.</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 344ms.</t>
+          <t>Load test on /api/medications completed. Response time: 231ms.</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 330ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 226ms.</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 440ms.</t>
+          <t>Load test on /api/login completed. Response time: 302ms.</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 348ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 168ms.</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 63ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 290ms.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 121ms.</t>
+          <t>Load test on /api/login completed. Response time: 227ms.</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 205ms.</t>
+          <t>Load test on /api/medications completed. Response time: 88ms.</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 198ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 348ms.</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 73ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 110ms.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 299ms.</t>
+          <t>Load test on /api/medications completed. Response time: 426ms.</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 400ms.</t>
+          <t>Load test on /api/medications completed. Response time: 76ms.</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 240ms.</t>
+          <t>Load test on /api/login completed. Response time: 152ms.</t>
         </is>
       </c>
     </row>
@@ -2184,17 +2184,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 364ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 739ms.</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 162ms.</t>
+          <t>Load test on /api/login completed. Response time: 56ms.</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 161ms.</t>
+          <t>Load test on /api/profile completed. Response time: 178ms.</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 99ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 53ms.</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 403ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 59ms.</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 393ms.</t>
+          <t>Load test on /api/medications completed. Response time: 63ms.</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 397ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 274ms.</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 405ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 334ms.</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 335ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 85ms.</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 334ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 351ms.</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 136ms.</t>
+          <t>Load test on /api/login completed. Response time: 144ms.</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 326ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 143ms.</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 429ms.</t>
+          <t>Load test on /api/login completed. Response time: 93ms.</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 80ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 291ms.</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 266ms.</t>
+          <t>Load test on /api/profile completed. Response time: 129ms.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 200ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 156ms.</t>
         </is>
       </c>
     </row>
@@ -2536,17 +2536,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 655ms.</t>
+          <t>Load test on /api/medications completed. Response time: 352ms.</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 353ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 387ms.</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 374ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 186ms.</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 332ms.</t>
+          <t>Load test on /api/medications completed. Response time: 96ms.</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 120ms.</t>
+          <t>Load test on /api/login completed. Response time: 306ms.</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 53ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 174ms.</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 421ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 224ms.</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 130ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 344ms.</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 360ms.</t>
+          <t>Load test on /api/medications completed. Response time: 127ms.</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 388ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 321ms.</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 210ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 415ms.</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 254ms.</t>
+          <t>Load test on /api/login completed. Response time: 325ms.</t>
         </is>
       </c>
     </row>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 212ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 394ms.</t>
         </is>
       </c>
     </row>
@@ -2822,17 +2822,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 1045ms.</t>
+          <t>Load test on /api/profile completed. Response time: 340ms.</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 428ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 348ms.</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 158ms.</t>
+          <t>Load test on /api/medications completed. Response time: 245ms.</t>
         </is>
       </c>
     </row>
@@ -2888,17 +2888,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 299ms.</t>
+          <t>Load test on /api/profile completed. Response time: 833ms.</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 435ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 253ms.</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 109ms.</t>
+          <t>Load test on /api/login completed. Response time: 179ms.</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 430ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 147ms.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 110ms.</t>
+          <t>Load test on /api/login completed. Response time: 375ms.</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 125ms.</t>
+          <t>Load test on /api/login completed. Response time: 97ms.</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 122ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 358ms.</t>
         </is>
       </c>
     </row>
@@ -3047,12 +3047,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 573ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 270ms.</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 443ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 56ms.</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 207ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 212ms.</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3108,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 88ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 172ms.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 384ms.</t>
+          <t>Load test on /api/login completed. Response time: 317ms.</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 262ms.</t>
+          <t>Load test on /api/medications completed. Response time: 420ms.</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 154ms.</t>
+          <t>Load test on /api/login completed. Response time: 428ms.</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 931ms.</t>
+          <t>Load test on /api/medications completed. Response time: 1432ms.</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 153ms.</t>
+          <t>Load test on /api/profile completed. Response time: 78ms.</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 149ms.</t>
+          <t>Load test on /api/profile completed. Response time: 332ms.</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 418ms.</t>
+          <t>Load test on /api/login completed. Response time: 182ms.</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 353ms.</t>
+          <t>Load test on /api/medications completed. Response time: 92ms.</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 172ms.</t>
+          <t>Load test on /api/medications completed. Response time: 132ms.</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 441ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 303ms.</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 444ms.</t>
+          <t>Load test on /api/login completed. Response time: 54ms.</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 192ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 99ms.</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 169ms.</t>
+          <t>Load test on /api/medications completed. Response time: 266ms.</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 202ms.</t>
+          <t>Load test on /api/profile completed. Response time: 239ms.</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 99ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 224ms.</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 345ms.</t>
+          <t>Load test on /api/login completed. Response time: 299ms.</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 231ms.</t>
+          <t>Load test on /api/login completed. Response time: 418ms.</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 254ms.</t>
+          <t>Load test on /api/medications completed. Response time: 267ms.</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 325ms.</t>
+          <t>Load test on /api/login completed. Response time: 320ms.</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 240ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 50ms.</t>
         </is>
       </c>
     </row>
@@ -3570,17 +3570,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 213ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 804ms.</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 65ms.</t>
+          <t>Load test on /api/login completed. Response time: 269ms.</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 94ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 190ms.</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 318ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 184ms.</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 355ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 95ms.</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 332ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 129ms.</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 439ms.</t>
+          <t>Load test on /api/login completed. Response time: 258ms.</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 324ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 436ms.</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 363ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 352ms.</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 94ms.</t>
+          <t>Load test on /api/login completed. Response time: 70ms.</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 216ms.</t>
+          <t>Load test on /api/login completed. Response time: 100ms.</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 345ms.</t>
+          <t>Load test on /api/medications completed. Response time: 395ms.</t>
         </is>
       </c>
     </row>
@@ -3834,17 +3834,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 646ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 333ms.</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 404ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 134ms.</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 362ms.</t>
+          <t>Load test on /api/medications completed. Response time: 114ms.</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 401ms.</t>
+          <t>Load test on /api/profile completed. Response time: 216ms.</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 252ms.</t>
+          <t>Load test on /api/login completed. Response time: 291ms.</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 225ms.</t>
+          <t>Load test on /api/medications completed. Response time: 101ms.</t>
         </is>
       </c>
     </row>
@@ -3966,17 +3966,17 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 383ms.</t>
+          <t>Load test on /api/medications completed. Response time: 1145ms.</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 260ms.</t>
+          <t>Load test on /api/profile completed. Response time: 299ms.</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 121ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 389ms.</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 445ms.</t>
+          <t>Load test on /api/profile completed. Response time: 205ms.</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 152ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 360ms.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 316ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 223ms.</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 52ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 409ms.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 184ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 101ms.</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 310ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 392ms.</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 296ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 92ms.</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 88ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 279ms.</t>
         </is>
       </c>
     </row>
@@ -4208,17 +4208,17 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 657ms.</t>
+          <t>Load test on /api/profile completed. Response time: 297ms.</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 274ms.</t>
+          <t>Load test on /api/medications completed. Response time: 413ms.</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 264ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 253ms.</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4274,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 360ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 119ms.</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 150ms.</t>
+          <t>Load test on /api/profile completed. Response time: 161ms.</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 51ms.</t>
+          <t>Load test on /api/login completed. Response time: 357ms.</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 196ms.</t>
+          <t>Load test on /api/login completed. Response time: 505ms.</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 332ms.</t>
+          <t>Load test on /api/login completed. Response time: 147ms.</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 339ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 332ms.</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 158ms.</t>
+          <t>Load test on /api/medications completed. Response time: 223ms.</t>
         </is>
       </c>
     </row>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 281ms.</t>
+          <t>Load test on /api/medications completed. Response time: 289ms.</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 356ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 329ms.</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 196ms.</t>
+          <t>Load test on /api/profile completed. Response time: 370ms.</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 135ms.</t>
+          <t>Load test on /api/medications completed. Response time: 162ms.</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 51ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 144ms.</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 289ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 355ms.</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 163ms.</t>
+          <t>Load test on /api/profile completed. Response time: 71ms.</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 63ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 212ms.</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 218ms.</t>
+          <t>Load test on /api/profile completed. Response time: 358ms.</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 583ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 883ms.</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 189ms.</t>
+          <t>Load test on /api/login completed. Response time: 217ms.</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 446ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 192ms.</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 158ms.</t>
+          <t>Load test on /api/medications completed. Response time: 71ms.</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 147ms.</t>
+          <t>Load test on /api/medications completed. Response time: 87ms.</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 91ms.</t>
+          <t>Load test on /api/login completed. Response time: 293ms.</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 426ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 183ms.</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 216ms.</t>
+          <t>Load test on /api/profile completed. Response time: 367ms.</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 338ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 238ms.</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 171ms.</t>
+          <t>Load test on /api/profile completed. Response time: 440ms.</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 216ms.</t>
+          <t>Load test on /api/medications completed. Response time: 291ms.</t>
         </is>
       </c>
     </row>
@@ -4868,17 +4868,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 395ms.</t>
+          <t>Load test on /api/profile completed. Response time: 1437ms.</t>
         </is>
       </c>
     </row>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 244ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 380ms.</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 192ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 402ms.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 328ms.</t>
+          <t>Load test on /api/profile completed. Response time: 236ms.</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 345ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 322ms.</t>
         </is>
       </c>
     </row>
@@ -4978,17 +4978,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 52ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 1001ms.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 414ms.</t>
+          <t>Load test on /api/profile completed. Response time: 276ms.</t>
         </is>
       </c>
     </row>
@@ -5022,17 +5022,17 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 904ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 104ms.</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 223ms.</t>
+          <t>Load test on /api/profile completed. Response time: 374ms.</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 165ms.</t>
+          <t>Load test on /api/medications completed. Response time: 317ms.</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 334ms.</t>
+          <t>Load test on /api/medications completed. Response time: 210ms.</t>
         </is>
       </c>
     </row>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 397ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 143ms.</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 444ms.</t>
+          <t>Load test on /api/profile completed. Response time: 225ms.</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 182ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 172ms.</t>
         </is>
       </c>
     </row>
@@ -5176,17 +5176,17 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 908ms.</t>
+          <t>Load test on /api/profile completed. Response time: 307ms.</t>
         </is>
       </c>
     </row>
@@ -5198,17 +5198,17 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 716ms.</t>
+          <t>Load test on /api/medications completed. Response time: 450ms.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 307ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 377ms.</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 730ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 1306ms.</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 226ms.</t>
+          <t>Load test on /api/login completed. Response time: 181ms.</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 150ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 300ms.</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5318,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 72ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 209ms.</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 260ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 355ms.</t>
         </is>
       </c>
     </row>
@@ -5362,7 +5362,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 366ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 441ms.</t>
         </is>
       </c>
     </row>
@@ -5374,7 +5374,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 258ms.</t>
+          <t>Load test on /api/profile completed. Response time: 116ms.</t>
         </is>
       </c>
     </row>
@@ -5396,17 +5396,17 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 244ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 970ms.</t>
         </is>
       </c>
     </row>
@@ -5418,17 +5418,17 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 1451ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 239ms.</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 135ms.</t>
+          <t>Load test on /api/medications completed. Response time: 135ms.</t>
         </is>
       </c>
     </row>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 335ms.</t>
+          <t>Load test on /api/medications completed. Response time: 408ms.</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 302ms.</t>
+          <t>Load test on /api/profile completed. Response time: 195ms.</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 391ms.</t>
+          <t>Load test on /api/profile completed. Response time: 236ms.</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 100ms.</t>
+          <t>Load test on /api/medications completed. Response time: 347ms.</t>
         </is>
       </c>
     </row>
@@ -5550,17 +5550,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 1151ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 433ms.</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 170ms.</t>
+          <t>Load test on /api/medications completed. Response time: 115ms.</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 91ms.</t>
+          <t>Load test on /api/profile completed. Response time: 223ms.</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 240ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 266ms.</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 276ms.</t>
+          <t>Load test on /api/login completed. Response time: 286ms.</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 216ms.</t>
+          <t>Load test on /api/profile completed. Response time: 116ms.</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 165ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 358ms.</t>
         </is>
       </c>
     </row>
@@ -5714,7 +5714,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 67ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 166ms.</t>
         </is>
       </c>
     </row>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 937ms.</t>
+          <t>Load test on /api/medications completed. Response time: 341ms.</t>
         </is>
       </c>
     </row>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 232ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 364ms.</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 304ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 94ms.</t>
         </is>
       </c>
     </row>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 196ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 324ms.</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 288ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 127ms.</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 199ms.</t>
+          <t>Load test on /api/medications completed. Response time: 110ms.</t>
         </is>
       </c>
     </row>
@@ -5868,7 +5868,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 217ms.</t>
+          <t>Load test on /api/profile completed. Response time: 336ms.</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5890,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 223ms.</t>
+          <t>Load test on /api/profile completed. Response time: 408ms.</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 267ms.</t>
+          <t>Load test on /api/medications completed. Response time: 289ms.</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 146ms.</t>
+          <t>Load test on /api/login completed. Response time: 323ms.</t>
         </is>
       </c>
     </row>
@@ -5946,7 +5946,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 415ms.</t>
+          <t>Load test on /api/medications completed. Response time: 257ms.</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 164ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 124ms.</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 109ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 90ms.</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 197ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 260ms.</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 285ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 180ms.</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 158ms.</t>
+          <t>Load test on /api/login completed. Response time: 148ms.</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6088,7 +6088,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 204ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 304ms.</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 136ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 232ms.</t>
         </is>
       </c>
     </row>
@@ -6122,17 +6122,17 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 595ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 145ms.</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 220ms.</t>
+          <t>Load test on /api/medications completed. Response time: 100ms.</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 323ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 188ms.</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 144ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 168ms.</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 219ms.</t>
+          <t>Load test on /api/medications completed. Response time: 147ms.</t>
         </is>
       </c>
     </row>
@@ -6237,12 +6237,12 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 221ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 1149ms.</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 155ms.</t>
+          <t>Load test on /api/medications completed. Response time: 349ms.</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 260ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 405ms.</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 251ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 60ms.</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 314ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 419ms.</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 450ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 161ms.</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 343ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 413ms.</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 396ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 90ms.</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 83ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 50ms.</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 83ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 117ms.</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 359ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 371ms.</t>
         </is>
       </c>
     </row>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 394ms.</t>
+          <t>Load test on /api/login completed. Response time: 239ms.</t>
         </is>
       </c>
     </row>
@@ -6496,7 +6496,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 152ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 245ms.</t>
         </is>
       </c>
     </row>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 420ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 278ms.</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 63ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 360ms.</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -6572,7 +6572,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 241ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 442ms.</t>
         </is>
       </c>
     </row>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 638ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 312ms.</t>
         </is>
       </c>
     </row>
@@ -6606,7 +6606,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/login</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Load test on /api/login completed. Response time: 245ms.</t>
+          <t>Load test on /api/medications completed. Response time: 197ms.</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 348ms.</t>
+          <t>Load test on /api/medications completed. Response time: 398ms.</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/medications</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 204ms.</t>
+          <t>Load test on /api/medications completed. Response time: 369ms.</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 437ms.</t>
+          <t>Load test on /api/login completed. Response time: 194ms.</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 417ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 88ms.</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 178ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 198ms.</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 117ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 76ms.</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 82ms.</t>
+          <t>Load test on /api/login completed. Response time: 332ms.</t>
         </is>
       </c>
     </row>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/profile</t>
+          <t>K6 Performance load test on /api/schedule</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 138ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 215ms.</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/metrics</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Load test on /api/metrics completed. Response time: 81ms.</t>
+          <t>Load test on /api/profile completed. Response time: 298ms.</t>
         </is>
       </c>
     </row>
@@ -6836,7 +6836,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 446ms.</t>
+          <t>Load test on /api/profile completed. Response time: 229ms.</t>
         </is>
       </c>
     </row>
@@ -6858,7 +6858,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 397ms.</t>
+          <t>Load test on /api/schedule completed. Response time: 215ms.</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6870,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 60ms.</t>
+          <t>Load test on /api/login completed. Response time: 145ms.</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 184ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 362ms.</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/vitals</t>
+          <t>K6 Performance load test on /api/login</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Load test on /api/vitals completed. Response time: 332ms.</t>
+          <t>Load test on /api/login completed. Response time: 217ms.</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 50ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 218ms.</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/schedule</t>
+          <t>K6 Performance load test on /api/vitals</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Load test on /api/schedule completed. Response time: 142ms.</t>
+          <t>Load test on /api/vitals completed. Response time: 380ms.</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/metrics</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 391ms.</t>
+          <t>Load test on /api/metrics completed. Response time: 400ms.</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>K6 Performance load test on /api/medications</t>
+          <t>K6 Performance load test on /api/profile</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Load test on /api/medications completed. Response time: 235ms.</t>
+          <t>Load test on /api/profile completed. Response time: 378ms.</t>
         </is>
       </c>
     </row>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Load test on /api/profile completed. Response time: 286ms.</t>
+          <t>Load test on /api/profile completed. Response time: 449ms.</t>
         </is>
       </c>
     </row>

</xml_diff>